<commit_message>
Cập nhật bài làm phần Hiển
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -477,185 +477,185 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Product — Tỷ lệ bản nháp đạt checklist chất lượng ngay lần QA đầu</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>T0: đo 20 bài gần nhất (chưa có số)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>≥80% ngày 60; ≥85% ngày 90</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Bảng QA mẫu 10 bài/tuần; brief + bản nháp + phiên bản cuối</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>An + QA content</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Mổ lỗi 5 bài; cập nhật prompt/checklist; giữ pilot</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
-        <is>
-          <t>Workflow — Thời gian từ brief hợp lệ đến bản nháp gửi QA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Workflow — Thời gian từ lúc brief được duyệt hợp lệ đến lúc bản nháp đầu tiên gửi QA (tính bằng giờ, lấy timestamp brief duyệt trừ timestamp gửi QA)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>workflow</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>T0: đo 10 brief hiện tại</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>≤70% baseline ngày 60</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="2">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Log timestamp brief/draft trong bảng theo dõi</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Chủ quy trình content</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Vẽ lại bước/handoff; hỗ trợ 1:1; chưa scale</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Product — Tỷ lệ claim/ý chính có nguồn kiểm chứng</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>T0: kiểm tra 20 bài</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>≥95% ngày 60</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Bảng QA đối chiếu brief/nguồn đã duyệt + link/version</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr" s="2">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Phụ trách QA content</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="2">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Chặn xuất bản; chuyển người duyệt claim; bổ sung nguồn</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Workflow — Tỷ lệ bản nháp phải sửa vì dài dòng/không bám brief</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>workflow</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>T0: phân loại 20 bài hiện tại</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>≤20% ngày 60; ≤15% ngày 90</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Phiếu QA + log vòng sửa</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Chủ quy trình content</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="2">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Bắt buộc dùng prompt template; xem lại brief và tiêu chí độ dài</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Workflow — Tỷ lệ chuyển người khi AI không chắc chắn/claim thiếu nguồn</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>workflow</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>T0: ghi trong pilot 30 ngày đầu</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>100% case rủi ro được chuyển; 0 claim chưa duyệt được xuất bản</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Log lỗi/flag + danh sách nội dung xuất bản</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="2">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Owner AI + người duyệt cuối</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="2">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Tạm dừng xuất bản; review nguyên nhân; cập nhật kho nguồn hoặc rule</t>
         </is>

</xml_diff>